<commit_message>
Actualizar evidencias con la paleta final y agregar tabla de SEO
</commit_message>
<xml_diff>
--- a/Accesibilidad_herramientas.xlsx
+++ b/Accesibilidad_herramientas.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="496" uniqueCount="289">
   <si>
     <t xml:space="preserve">Accesibilidad – Herramientas de trabajo</t>
   </si>
@@ -210,10 +210,10 @@
     <t xml:space="preserve">Evidencias_accesibilidad/07_contraste/tabla_de_contraste_paleta.png</t>
   </si>
   <si>
-    <t xml:space="preserve">La paleta bordó #6C0808 / crema #F0E9D7 tiene contraste 10.35:1; texto principal 14.7:1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Se corrigieron migas de pan y contador de resultados de WooCommerce (2.7:1 → 7.8:1).</t>
+    <t xml:space="preserve">Paleta Valten: párrafos #2D0000 sobre #F0E9D7 = 15.6:1; títulos #6C0808 sobre #F0E9D7 = 10.35:1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El verde #757D6E (3.53:1) se usa solo en líneas, bordes y detalles gráficos, nunca en texto chico.</t>
   </si>
   <si>
     <t xml:space="preserve">Contraste de botones y campos</t>
@@ -231,10 +231,10 @@
     <t xml:space="preserve">Corregido</t>
   </si>
   <si>
-    <t xml:space="preserve">Botones, bordes de campos (5.4:1) e indicador de foco superan 3:1.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">El aviso azul de 'agregado al carrito' (2.7:1) se cambió a crema con borde bordó.</t>
+    <t xml:space="preserve">Botones (beige sobre bordó 10.35:1), bordes verdes de tarjetas y campos (3.53:1) e indicador de foco superan 3:1.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se corrigió el botón 'Pasar al pago' del carrito (1.04:1 → 10.35:1) y el aviso de 'agregado al carrito'.</t>
   </si>
   <si>
     <t xml:space="preserve">Navegación por teclado</t>
@@ -255,7 +255,7 @@
     <t xml:space="preserve">Evidencias_accesibilidad/05_prueba_teclado/</t>
   </si>
   <si>
-    <t xml:space="preserve">Se recorrió Inicio → Tienda → ficha → Agregar al carrito → Carrito → Finalizar compra → Contacto solo con Tab y Enter.</t>
+    <t xml:space="preserve">Se recorrió Inicio → Tienda → ficha → Agregar al carrito → Carrito (Pasar al pago) → Checkout → Contacto solo con Tab y Enter.</t>
   </si>
   <si>
     <t xml:space="preserve">Se agregaron nombre y control por teclado al buscador y al botón de menú del header.</t>
@@ -282,7 +282,7 @@
     <t xml:space="preserve">Cada enlace, botón y campo muestra un indicador al recibir el foco.</t>
   </si>
   <si>
-    <t xml:space="preserve">Evidencias_accesibilidad/05_prueba_teclado/04_ficha_foco_agregar_al_carrito.png</t>
+    <t xml:space="preserve">Evidencias_accesibilidad/05_prueba_teclado/06_carrito_foco_pasar_al_pago.png</t>
   </si>
   <si>
     <t xml:space="preserve">Cada enlace, botón y campo muestra un contorno bordó de 3 px al recibir el foco.</t>
@@ -393,10 +393,10 @@
     <t xml:space="preserve">Evidencias_accesibilidad/08_auditoria_automatica/informe_antes_despues.png</t>
   </si>
   <si>
-    <t xml:space="preserve">Auditoría automática con axe-core: 143 elementos con problemas antes, 10 después.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Los 10 restantes son componentes internos de WooCommerce.</t>
+    <t xml:space="preserve">Auditoría automática con axe-core: 143 elementos con problemas antes, 5 después.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los restantes son componentes internos de WooCommerce (aviso del carrito y animación de carga).</t>
   </si>
   <si>
     <t xml:space="preserve">Mensajes de error claros</t>
@@ -633,7 +633,7 @@
     <t xml:space="preserve">Promedio / Total</t>
   </si>
   <si>
-    <t xml:space="preserve">Frase para el PDF/video: "La auditoría automática bajó de 143 a 10 elementos con problemas en todo el sitio (29 a 2 en las 5 páginas principales)."</t>
+    <t xml:space="preserve">Frase para el PDF/video: "La auditoría automática bajó de 143 a 5 elementos con problemas en todo el sitio (29 a 2 en las 5 páginas principales)."</t>
   </si>
   <si>
     <t xml:space="preserve">Registro de trabajo – Especialista en accesibilidad</t>
@@ -760,6 +760,12 @@
   </si>
   <si>
     <t xml:space="preserve">10 elementos pendientes, todos internos de WooCommerce.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nueva validación tras el cambio de paleta y tipografía del sitio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contraste verificado con la paleta final; auditoría final: 5 elementos pendientes (internos de WooCommerce).</t>
   </si>
   <si>
     <t xml:space="preserve">Pendiente</t>
@@ -2612,11 +2618,11 @@
         <v>12</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E8" s="18" t="n">
         <f aca="false">IF(OR(C8="",D8=""),"",C8-D8)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F8" s="15"/>
       <c r="G8" s="15"/>
@@ -2640,11 +2646,11 @@
         <v>5</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E9" s="18" t="n">
         <f aca="false">IF(OR(C9="",D9=""),"",C9-D9)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F9" s="15"/>
       <c r="G9" s="15"/>
@@ -3000,14 +3006,26 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="16"/>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+      <c r="A13" s="16" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>59</v>
+      </c>
       <c r="G13" s="15" t="s">
-        <v>244</v>
+        <v>214</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3018,7 +3036,7 @@
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
       <c r="G14" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3029,7 +3047,7 @@
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
       <c r="G15" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3040,7 +3058,7 @@
       <c r="E16" s="15"/>
       <c r="F16" s="15"/>
       <c r="G16" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3051,7 +3069,7 @@
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
       <c r="G17" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3062,7 +3080,7 @@
       <c r="E18" s="15"/>
       <c r="F18" s="15"/>
       <c r="G18" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3073,7 +3091,7 @@
       <c r="E19" s="15"/>
       <c r="F19" s="15"/>
       <c r="G19" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3084,7 +3102,7 @@
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
       <c r="G20" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3095,7 +3113,7 @@
       <c r="E21" s="15"/>
       <c r="F21" s="15"/>
       <c r="G21" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3106,7 +3124,7 @@
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
       <c r="G22" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3117,7 +3135,7 @@
       <c r="E23" s="15"/>
       <c r="F23" s="15"/>
       <c r="G23" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3128,7 +3146,7 @@
       <c r="E24" s="15"/>
       <c r="F24" s="15"/>
       <c r="G24" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3139,7 +3157,7 @@
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
       <c r="G25" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3150,7 +3168,7 @@
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
       <c r="G26" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3161,7 +3179,7 @@
       <c r="E27" s="15"/>
       <c r="F27" s="15"/>
       <c r="G27" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3172,7 +3190,7 @@
       <c r="E28" s="15"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3183,7 +3201,7 @@
       <c r="E29" s="15"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3194,7 +3212,7 @@
       <c r="E30" s="15"/>
       <c r="F30" s="15"/>
       <c r="G30" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3205,7 +3223,7 @@
       <c r="E31" s="15"/>
       <c r="F31" s="15"/>
       <c r="G31" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3216,7 +3234,7 @@
       <c r="E32" s="15"/>
       <c r="F32" s="15"/>
       <c r="G32" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3227,7 +3245,7 @@
       <c r="E33" s="15"/>
       <c r="F33" s="15"/>
       <c r="G33" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3238,7 +3256,7 @@
       <c r="E34" s="15"/>
       <c r="F34" s="15"/>
       <c r="G34" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3249,7 +3267,7 @@
       <c r="E35" s="15"/>
       <c r="F35" s="15"/>
       <c r="G35" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3260,7 +3278,7 @@
       <c r="E36" s="15"/>
       <c r="F36" s="15"/>
       <c r="G36" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3271,7 +3289,7 @@
       <c r="E37" s="15"/>
       <c r="F37" s="15"/>
       <c r="G37" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3282,7 +3300,7 @@
       <c r="E38" s="15"/>
       <c r="F38" s="15"/>
       <c r="G38" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3293,7 +3311,7 @@
       <c r="E39" s="15"/>
       <c r="F39" s="15"/>
       <c r="G39" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3304,7 +3322,7 @@
       <c r="E40" s="15"/>
       <c r="F40" s="15"/>
       <c r="G40" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3352,12 +3370,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="B2" s="6" t="str">
         <f aca="false">COUNTIF(D5:D35,"Completada")&amp;" de "&amp;COUNTA(B5:B35)&amp;" tareas completadas ("&amp;TEXT(COUNTIF(D5:D35,"Completada")/COUNTA(B5:B35),"0%")&amp;")"</f>
@@ -3366,10 +3384,10 @@
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>36</v>
@@ -3380,52 +3398,52 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C5" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C6" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C7" s="14" t="s">
         <v>125</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C8" s="14" t="s">
         <v>125</v>
@@ -3436,10 +3454,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C9" s="14" t="s">
         <v>46</v>
@@ -3450,10 +3468,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C10" s="14" t="s">
         <v>46</v>
@@ -3464,10 +3482,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C11" s="14" t="s">
         <v>46</v>
@@ -3478,10 +3496,10 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B12" s="14" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C12" s="14" t="s">
         <v>46</v>
@@ -3492,10 +3510,10 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="C13" s="14" t="s">
         <v>46</v>
@@ -3506,10 +3524,10 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C14" s="14" t="s">
         <v>46</v>
@@ -3520,10 +3538,10 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C15" s="14" t="s">
         <v>46</v>
@@ -3534,10 +3552,10 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>125</v>
@@ -3548,10 +3566,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="C17" s="14" t="s">
         <v>125</v>
@@ -3562,10 +3580,10 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C18" s="14" t="s">
         <v>125</v>
@@ -3576,24 +3594,24 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C19" s="14" t="s">
         <v>125</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C20" s="14" t="s">
         <v>46</v>
@@ -3604,24 +3622,24 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C22" s="14" t="s">
         <v>46</v>
@@ -3632,10 +3650,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C23" s="14" t="s">
         <v>46</v>
@@ -3646,10 +3664,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C24" s="14" t="s">
         <v>125</v>
@@ -3660,10 +3678,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C25" s="14" t="s">
         <v>46</v>
@@ -3674,142 +3692,142 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C26" s="14" t="s">
         <v>125</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C27" s="14" t="s">
         <v>125</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C29" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C30" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="C31" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B32" s="14" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C32" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B33" s="14" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C33" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B34" s="14" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="C34" s="14" t="s">
         <v>46</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C35" s="14" t="s">
         <v>125</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
   </sheetData>

</xml_diff>